<commit_message>
#9 Client BOM Updated
</commit_message>
<xml_diff>
--- a/BOM/Client-BOM.xlsx
+++ b/BOM/Client-BOM.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="859" uniqueCount="277">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="927" uniqueCount="309">
   <si>
     <t>Component list</t>
   </si>
@@ -851,6 +851,102 @@
   </si>
   <si>
     <t>TS-1109S-C-B</t>
+  </si>
+  <si>
+    <t>C1, C2, C3, C4</t>
+  </si>
+  <si>
+    <t>CAP CER 1000PF 25V C0G 0402</t>
+  </si>
+  <si>
+    <t>C1005C0G1E102JT000F</t>
+  </si>
+  <si>
+    <t>TDK</t>
+  </si>
+  <si>
+    <t>1nF</t>
+  </si>
+  <si>
+    <t>C62</t>
+  </si>
+  <si>
+    <t>D1</t>
+  </si>
+  <si>
+    <t>TVS DIODE 5VWM 6.3VC DSN0603-2</t>
+  </si>
+  <si>
+    <t>DSN0603-2</t>
+  </si>
+  <si>
+    <t>PESD5V0H1BSFYL</t>
+  </si>
+  <si>
+    <t>Nexperia</t>
+  </si>
+  <si>
+    <t>Fuse</t>
+  </si>
+  <si>
+    <t>F1</t>
+  </si>
+  <si>
+    <t>6V 2A 50A 1W -40℃~+85℃ 4A 4mΩ 5s 45mΩ 0805 Resettable Fuses ROHS</t>
+  </si>
+  <si>
+    <t>Fuse-0805</t>
+  </si>
+  <si>
+    <t>BSMD0805L-200</t>
+  </si>
+  <si>
+    <t>BHFUSE</t>
+  </si>
+  <si>
+    <t>USB Connector</t>
+  </si>
+  <si>
+    <t>J2</t>
+  </si>
+  <si>
+    <t>USB 3.1 1 Brick nogging 16 Female Type-C SMD USB Connectors ROHS</t>
+  </si>
+  <si>
+    <t>918-418K2022Y40009</t>
+  </si>
+  <si>
+    <t>Jing Extension</t>
+  </si>
+  <si>
+    <t>R1, R2</t>
+  </si>
+  <si>
+    <t>RES 5.1K OHM 1% 1/16W 0402</t>
+  </si>
+  <si>
+    <t>Res-0402</t>
+  </si>
+  <si>
+    <t>RC0402FR-075K1L</t>
+  </si>
+  <si>
+    <t>5.1K</t>
+  </si>
+  <si>
+    <t>SW1</t>
+  </si>
+  <si>
+    <t>-25℃~+85℃ 6mm 5mm Round Button 50mA Brick nogging 6mm SPST 100MΩ 100000 250gf@±30gf 12V SMD Tactile Switches ROHS</t>
+  </si>
+  <si>
+    <t>K2-1102SP-C4SC-04</t>
+  </si>
+  <si>
+    <t>Korean Hroparts Elec</t>
+  </si>
+  <si>
+    <t>SIDE PCB BOM</t>
   </si>
 </sst>
 </file>
@@ -861,7 +957,7 @@
     <numFmt numFmtId="164" formatCode="[$-409]h:mm:ss\ AM/PM;@"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.0000"/>
   </numFmts>
-  <fonts count="24" x14ac:knownFonts="1">
+  <fonts count="26" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1026,6 +1122,21 @@
       <b/>
       <sz val="10"/>
       <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1312,7 +1423,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="82">
+  <cellXfs count="87">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1469,24 +1580,6 @@
     <xf numFmtId="0" fontId="18" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="17" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1532,6 +1625,39 @@
     </xf>
     <xf numFmtId="0" fontId="23" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1927,7 +2053,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L81"/>
+  <dimension ref="A1:L82"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3" bestFit="1" customWidth="1"/>
@@ -1952,10 +2078,10 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="60"/>
-      <c r="J1" s="60"/>
-      <c r="K1" s="60"/>
-      <c r="L1" s="61"/>
+      <c r="I1" s="76"/>
+      <c r="J1" s="76"/>
+      <c r="K1" s="76"/>
+      <c r="L1" s="77"/>
     </row>
     <row r="2" spans="1:12" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -1991,7 +2117,7 @@
       <c r="I3" s="5"/>
       <c r="J3" s="5"/>
       <c r="K3" s="5"/>
-      <c r="L3" s="62"/>
+      <c r="L3" s="78"/>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -2009,7 +2135,7 @@
       <c r="I4" s="7"/>
       <c r="J4" s="6"/>
       <c r="K4" s="6"/>
-      <c r="L4" s="63"/>
+      <c r="L4" s="79"/>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -2027,7 +2153,7 @@
       <c r="I5" s="6"/>
       <c r="J5" s="6"/>
       <c r="K5" s="6"/>
-      <c r="L5" s="63"/>
+      <c r="L5" s="79"/>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -2041,7 +2167,7 @@
       <c r="I6" s="6"/>
       <c r="J6" s="6"/>
       <c r="K6" s="6"/>
-      <c r="L6" s="63"/>
+      <c r="L6" s="79"/>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -2055,7 +2181,7 @@
       <c r="I7" s="8"/>
       <c r="J7" s="8"/>
       <c r="K7" s="8"/>
-      <c r="L7" s="63"/>
+      <c r="L7" s="79"/>
     </row>
     <row r="8" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -2069,7 +2195,7 @@
       <c r="I8" s="8"/>
       <c r="J8" s="8"/>
       <c r="K8" s="8"/>
-      <c r="L8" s="63"/>
+      <c r="L8" s="79"/>
     </row>
     <row r="9" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -2100,7 +2226,7 @@
       <c r="J9" s="27" t="s">
         <v>221</v>
       </c>
-      <c r="K9" s="66" t="s">
+      <c r="K9" s="60" t="s">
         <v>228</v>
       </c>
       <c r="L9" s="27" t="s">
@@ -2137,7 +2263,7 @@
       <c r="J10" s="33">
         <v>3</v>
       </c>
-      <c r="K10" s="67"/>
+      <c r="K10" s="61"/>
       <c r="L10" s="51"/>
     </row>
     <row r="11" spans="1:12" s="52" customFormat="1" x14ac:dyDescent="0.25">
@@ -2170,7 +2296,7 @@
       <c r="J11" s="36">
         <v>2</v>
       </c>
-      <c r="K11" s="68"/>
+      <c r="K11" s="62"/>
       <c r="L11" s="36"/>
     </row>
     <row r="12" spans="1:12" s="52" customFormat="1" ht="24" x14ac:dyDescent="0.25">
@@ -2203,7 +2329,7 @@
       <c r="J12" s="33">
         <v>14</v>
       </c>
-      <c r="K12" s="67"/>
+      <c r="K12" s="61"/>
       <c r="L12" s="40"/>
     </row>
     <row r="13" spans="1:12" s="52" customFormat="1" x14ac:dyDescent="0.25">
@@ -2236,7 +2362,7 @@
       <c r="J13" s="36">
         <v>1</v>
       </c>
-      <c r="K13" s="68"/>
+      <c r="K13" s="62"/>
       <c r="L13" s="40"/>
     </row>
     <row r="14" spans="1:12" s="52" customFormat="1" ht="36" x14ac:dyDescent="0.25">
@@ -2269,7 +2395,7 @@
       <c r="J14" s="33">
         <v>22</v>
       </c>
-      <c r="K14" s="67"/>
+      <c r="K14" s="61"/>
       <c r="L14" s="40"/>
     </row>
     <row r="15" spans="1:12" s="52" customFormat="1" x14ac:dyDescent="0.25">
@@ -2302,7 +2428,7 @@
       <c r="J15" s="36">
         <v>2</v>
       </c>
-      <c r="K15" s="68"/>
+      <c r="K15" s="62"/>
       <c r="L15" s="40"/>
     </row>
     <row r="16" spans="1:12" s="52" customFormat="1" x14ac:dyDescent="0.25">
@@ -2335,7 +2461,7 @@
       <c r="J16" s="33">
         <v>2</v>
       </c>
-      <c r="K16" s="67"/>
+      <c r="K16" s="61"/>
       <c r="L16" s="40"/>
     </row>
     <row r="17" spans="1:12" s="52" customFormat="1" x14ac:dyDescent="0.25">
@@ -2368,7 +2494,7 @@
       <c r="J17" s="36">
         <v>6</v>
       </c>
-      <c r="K17" s="68"/>
+      <c r="K17" s="62"/>
       <c r="L17" s="40"/>
     </row>
     <row r="18" spans="1:12" s="52" customFormat="1" x14ac:dyDescent="0.25">
@@ -2401,7 +2527,7 @@
       <c r="J18" s="33">
         <v>3</v>
       </c>
-      <c r="K18" s="67"/>
+      <c r="K18" s="61"/>
       <c r="L18" s="40"/>
     </row>
     <row r="19" spans="1:12" s="52" customFormat="1" x14ac:dyDescent="0.25">
@@ -2434,7 +2560,7 @@
       <c r="J19" s="36">
         <v>1</v>
       </c>
-      <c r="K19" s="68"/>
+      <c r="K19" s="62"/>
       <c r="L19" s="40"/>
     </row>
     <row r="20" spans="1:12" s="52" customFormat="1" x14ac:dyDescent="0.25">
@@ -2467,7 +2593,7 @@
       <c r="J20" s="36">
         <v>2</v>
       </c>
-      <c r="K20" s="68"/>
+      <c r="K20" s="62"/>
       <c r="L20" s="40"/>
     </row>
     <row r="21" spans="1:12" s="52" customFormat="1" x14ac:dyDescent="0.25">
@@ -2500,7 +2626,7 @@
       <c r="J21" s="33">
         <v>2</v>
       </c>
-      <c r="K21" s="67"/>
+      <c r="K21" s="61"/>
       <c r="L21" s="40"/>
     </row>
     <row r="22" spans="1:12" s="52" customFormat="1" x14ac:dyDescent="0.25">
@@ -2533,7 +2659,7 @@
       <c r="J22" s="36">
         <v>1</v>
       </c>
-      <c r="K22" s="68"/>
+      <c r="K22" s="62"/>
       <c r="L22" s="40"/>
     </row>
     <row r="23" spans="1:12" s="52" customFormat="1" ht="24" x14ac:dyDescent="0.25">
@@ -2566,7 +2692,7 @@
       <c r="J23" s="36">
         <v>1</v>
       </c>
-      <c r="K23" s="68"/>
+      <c r="K23" s="62"/>
       <c r="L23" s="40"/>
     </row>
     <row r="24" spans="1:12" s="52" customFormat="1" ht="24" x14ac:dyDescent="0.25">
@@ -2599,7 +2725,7 @@
       <c r="J24" s="33">
         <v>1</v>
       </c>
-      <c r="K24" s="67"/>
+      <c r="K24" s="61"/>
       <c r="L24" s="40"/>
     </row>
     <row r="25" spans="1:12" s="52" customFormat="1" ht="24" x14ac:dyDescent="0.25">
@@ -2632,7 +2758,7 @@
       <c r="J25" s="36">
         <v>1</v>
       </c>
-      <c r="K25" s="69"/>
+      <c r="K25" s="63"/>
       <c r="L25" s="36"/>
     </row>
     <row r="26" spans="1:12" s="52" customFormat="1" ht="24" x14ac:dyDescent="0.25">
@@ -2665,7 +2791,7 @@
       <c r="J26" s="33">
         <v>2</v>
       </c>
-      <c r="K26" s="67"/>
+      <c r="K26" s="61"/>
       <c r="L26" s="40"/>
     </row>
     <row r="27" spans="1:12" s="52" customFormat="1" ht="24" x14ac:dyDescent="0.25">
@@ -2698,7 +2824,7 @@
       <c r="J27" s="36">
         <v>1</v>
       </c>
-      <c r="K27" s="68"/>
+      <c r="K27" s="62"/>
       <c r="L27" s="40"/>
     </row>
     <row r="28" spans="1:12" s="52" customFormat="1" x14ac:dyDescent="0.25">
@@ -2731,7 +2857,7 @@
       <c r="J28" s="43">
         <v>1</v>
       </c>
-      <c r="K28" s="70"/>
+      <c r="K28" s="64"/>
       <c r="L28" s="46"/>
     </row>
     <row r="29" spans="1:12" s="52" customFormat="1" ht="48" x14ac:dyDescent="0.25">
@@ -2764,7 +2890,7 @@
       <c r="J29" s="36">
         <v>3</v>
       </c>
-      <c r="K29" s="68"/>
+      <c r="K29" s="62"/>
       <c r="L29" s="40"/>
     </row>
     <row r="30" spans="1:12" s="52" customFormat="1" ht="24" x14ac:dyDescent="0.25">
@@ -2797,7 +2923,7 @@
       <c r="J30" s="33">
         <v>1</v>
       </c>
-      <c r="K30" s="71" t="s">
+      <c r="K30" s="65" t="s">
         <v>273</v>
       </c>
       <c r="L30" s="40"/>
@@ -2832,7 +2958,7 @@
       <c r="J31" s="36">
         <v>1</v>
       </c>
-      <c r="K31" s="68"/>
+      <c r="K31" s="62"/>
       <c r="L31" s="40"/>
     </row>
     <row r="32" spans="1:12" s="52" customFormat="1" ht="48" x14ac:dyDescent="0.25">
@@ -2865,7 +2991,7 @@
       <c r="J32" s="33">
         <v>1</v>
       </c>
-      <c r="K32" s="67"/>
+      <c r="K32" s="61"/>
       <c r="L32" s="40"/>
     </row>
     <row r="33" spans="1:12" s="52" customFormat="1" x14ac:dyDescent="0.25">
@@ -2898,7 +3024,7 @@
       <c r="J33" s="36">
         <v>1</v>
       </c>
-      <c r="K33" s="68"/>
+      <c r="K33" s="62"/>
       <c r="L33" s="40"/>
     </row>
     <row r="34" spans="1:12" s="52" customFormat="1" ht="24" x14ac:dyDescent="0.25">
@@ -2931,7 +3057,7 @@
       <c r="J34" s="43">
         <v>13</v>
       </c>
-      <c r="K34" s="70"/>
+      <c r="K34" s="64"/>
       <c r="L34" s="46"/>
     </row>
     <row r="35" spans="1:12" s="52" customFormat="1" ht="36" x14ac:dyDescent="0.25">
@@ -2964,7 +3090,7 @@
       <c r="J35" s="36">
         <v>1</v>
       </c>
-      <c r="K35" s="68"/>
+      <c r="K35" s="62"/>
       <c r="L35" s="40"/>
     </row>
     <row r="36" spans="1:12" s="52" customFormat="1" x14ac:dyDescent="0.25">
@@ -2997,7 +3123,7 @@
       <c r="J36" s="33">
         <v>1</v>
       </c>
-      <c r="K36" s="67"/>
+      <c r="K36" s="61"/>
       <c r="L36" s="40"/>
     </row>
     <row r="37" spans="1:12" s="52" customFormat="1" ht="48" x14ac:dyDescent="0.25">
@@ -3030,7 +3156,7 @@
       <c r="J37" s="36">
         <v>11</v>
       </c>
-      <c r="K37" s="72" t="s">
+      <c r="K37" s="66" t="s">
         <v>235</v>
       </c>
       <c r="L37" s="40"/>
@@ -3065,7 +3191,7 @@
       <c r="J38" s="36">
         <v>3</v>
       </c>
-      <c r="K38" s="68"/>
+      <c r="K38" s="62"/>
       <c r="L38" s="40"/>
     </row>
     <row r="39" spans="1:12" s="52" customFormat="1" x14ac:dyDescent="0.25">
@@ -3098,7 +3224,7 @@
       <c r="J39" s="36">
         <v>1</v>
       </c>
-      <c r="K39" s="67"/>
+      <c r="K39" s="61"/>
       <c r="L39" s="40"/>
     </row>
     <row r="40" spans="1:12" s="52" customFormat="1" x14ac:dyDescent="0.25">
@@ -3131,7 +3257,7 @@
       <c r="J40" s="33">
         <v>2</v>
       </c>
-      <c r="K40" s="67"/>
+      <c r="K40" s="61"/>
       <c r="L40" s="40"/>
     </row>
     <row r="41" spans="1:12" s="52" customFormat="1" ht="36" x14ac:dyDescent="0.25">
@@ -3164,7 +3290,7 @@
       <c r="J41" s="36">
         <v>1</v>
       </c>
-      <c r="K41" s="68"/>
+      <c r="K41" s="62"/>
       <c r="L41" s="40"/>
     </row>
     <row r="42" spans="1:12" s="52" customFormat="1" x14ac:dyDescent="0.25">
@@ -3197,7 +3323,7 @@
       <c r="J42" s="33">
         <v>5</v>
       </c>
-      <c r="K42" s="67"/>
+      <c r="K42" s="61"/>
       <c r="L42" s="40"/>
     </row>
     <row r="43" spans="1:12" s="52" customFormat="1" x14ac:dyDescent="0.25">
@@ -3230,7 +3356,7 @@
       <c r="J43" s="36">
         <v>2</v>
       </c>
-      <c r="K43" s="68"/>
+      <c r="K43" s="62"/>
       <c r="L43" s="40"/>
     </row>
     <row r="44" spans="1:12" s="52" customFormat="1" x14ac:dyDescent="0.25">
@@ -3263,7 +3389,7 @@
       <c r="J44" s="33">
         <v>3</v>
       </c>
-      <c r="K44" s="67"/>
+      <c r="K44" s="61"/>
       <c r="L44" s="40"/>
     </row>
     <row r="45" spans="1:12" s="52" customFormat="1" x14ac:dyDescent="0.25">
@@ -3296,7 +3422,7 @@
       <c r="J45" s="36">
         <v>2</v>
       </c>
-      <c r="K45" s="68"/>
+      <c r="K45" s="62"/>
       <c r="L45" s="40"/>
     </row>
     <row r="46" spans="1:12" s="52" customFormat="1" x14ac:dyDescent="0.25">
@@ -3329,41 +3455,41 @@
       <c r="J46" s="33">
         <v>2</v>
       </c>
-      <c r="K46" s="67"/>
+      <c r="K46" s="61"/>
       <c r="L46" s="40"/>
     </row>
     <row r="47" spans="1:12" s="52" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="73"/>
-      <c r="B47" s="74">
+      <c r="A47" s="67"/>
+      <c r="B47" s="68">
         <f t="shared" si="0"/>
         <v>38</v>
       </c>
-      <c r="C47" s="75" t="s">
+      <c r="C47" s="69" t="s">
         <v>15</v>
       </c>
-      <c r="D47" s="76" t="s">
+      <c r="D47" s="70" t="s">
         <v>51</v>
       </c>
-      <c r="E47" s="76" t="s">
+      <c r="E47" s="70" t="s">
         <v>96</v>
       </c>
-      <c r="F47" s="76" t="s">
+      <c r="F47" s="70" t="s">
         <v>123</v>
       </c>
-      <c r="G47" s="76" t="s">
+      <c r="G47" s="70" t="s">
         <v>163</v>
       </c>
-      <c r="H47" s="76" t="s">
+      <c r="H47" s="70" t="s">
         <v>177</v>
       </c>
-      <c r="I47" s="76" t="s">
+      <c r="I47" s="70" t="s">
         <v>219</v>
       </c>
-      <c r="J47" s="76">
-        <v>1</v>
-      </c>
-      <c r="K47" s="77"/>
-      <c r="L47" s="78"/>
+      <c r="J47" s="70">
+        <v>1</v>
+      </c>
+      <c r="K47" s="71"/>
+      <c r="L47" s="72"/>
     </row>
     <row r="48" spans="1:12" s="52" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A48" s="50"/>
@@ -3395,7 +3521,7 @@
       <c r="J48" s="33">
         <v>1</v>
       </c>
-      <c r="K48" s="67"/>
+      <c r="K48" s="61"/>
       <c r="L48" s="40"/>
     </row>
     <row r="49" spans="1:12" s="52" customFormat="1" x14ac:dyDescent="0.25">
@@ -3428,7 +3554,7 @@
       <c r="J49" s="43">
         <v>6</v>
       </c>
-      <c r="K49" s="70"/>
+      <c r="K49" s="64"/>
       <c r="L49" s="46"/>
     </row>
     <row r="50" spans="1:12" s="52" customFormat="1" ht="48" x14ac:dyDescent="0.25">
@@ -3461,7 +3587,7 @@
       <c r="J50" s="36">
         <v>2</v>
       </c>
-      <c r="K50" s="72"/>
+      <c r="K50" s="66"/>
       <c r="L50" s="36"/>
     </row>
     <row r="51" spans="1:12" ht="36" x14ac:dyDescent="0.25">
@@ -3494,7 +3620,7 @@
       <c r="J51" s="33">
         <v>1</v>
       </c>
-      <c r="K51" s="79"/>
+      <c r="K51" s="73"/>
       <c r="L51" s="33"/>
     </row>
     <row r="52" spans="1:12" s="52" customFormat="1" ht="48" x14ac:dyDescent="0.25">
@@ -3527,7 +3653,7 @@
       <c r="J52" s="36">
         <v>1</v>
       </c>
-      <c r="K52" s="68"/>
+      <c r="K52" s="62"/>
       <c r="L52" s="40"/>
     </row>
     <row r="53" spans="1:12" s="52" customFormat="1" ht="24" x14ac:dyDescent="0.25">
@@ -3560,7 +3686,7 @@
       <c r="J53" s="33">
         <v>1</v>
       </c>
-      <c r="K53" s="67"/>
+      <c r="K53" s="61"/>
       <c r="L53" s="40"/>
     </row>
     <row r="54" spans="1:12" s="52" customFormat="1" x14ac:dyDescent="0.25">
@@ -3593,7 +3719,7 @@
       <c r="J54" s="36">
         <v>1</v>
       </c>
-      <c r="K54" s="68"/>
+      <c r="K54" s="62"/>
       <c r="L54" s="40"/>
     </row>
     <row r="55" spans="1:12" s="52" customFormat="1" ht="24" x14ac:dyDescent="0.25">
@@ -3626,7 +3752,7 @@
       <c r="J55" s="33">
         <v>1</v>
       </c>
-      <c r="K55" s="67"/>
+      <c r="K55" s="61"/>
       <c r="L55" s="40"/>
     </row>
     <row r="56" spans="1:12" s="52" customFormat="1" ht="24" x14ac:dyDescent="0.25">
@@ -3659,7 +3785,7 @@
       <c r="J56" s="36">
         <v>1</v>
       </c>
-      <c r="K56" s="68"/>
+      <c r="K56" s="62"/>
       <c r="L56" s="40"/>
     </row>
     <row r="57" spans="1:12" s="52" customFormat="1" ht="24" x14ac:dyDescent="0.25">
@@ -3692,7 +3818,7 @@
       <c r="J57" s="33">
         <v>1</v>
       </c>
-      <c r="K57" s="67"/>
+      <c r="K57" s="61"/>
       <c r="L57" s="40"/>
     </row>
     <row r="58" spans="1:12" s="52" customFormat="1" ht="24" x14ac:dyDescent="0.25">
@@ -3725,7 +3851,7 @@
       <c r="J58" s="33">
         <v>1</v>
       </c>
-      <c r="K58" s="67"/>
+      <c r="K58" s="61"/>
       <c r="L58" s="40"/>
     </row>
     <row r="59" spans="1:12" s="52" customFormat="1" ht="24" x14ac:dyDescent="0.25">
@@ -3758,7 +3884,7 @@
       <c r="J59" s="36">
         <v>1</v>
       </c>
-      <c r="K59" s="68"/>
+      <c r="K59" s="62"/>
       <c r="L59" s="40"/>
     </row>
     <row r="60" spans="1:12" s="52" customFormat="1" ht="24" x14ac:dyDescent="0.25">
@@ -3791,7 +3917,7 @@
       <c r="J60" s="33">
         <v>1</v>
       </c>
-      <c r="K60" s="67"/>
+      <c r="K60" s="61"/>
       <c r="L60" s="40"/>
     </row>
     <row r="61" spans="1:12" s="52" customFormat="1" x14ac:dyDescent="0.25">
@@ -3824,7 +3950,7 @@
       <c r="J61" s="36">
         <v>1</v>
       </c>
-      <c r="K61" s="68"/>
+      <c r="K61" s="62"/>
       <c r="L61" s="40"/>
     </row>
     <row r="62" spans="1:12" s="52" customFormat="1" ht="24" x14ac:dyDescent="0.25">
@@ -3857,7 +3983,7 @@
       <c r="J62" s="33">
         <v>1</v>
       </c>
-      <c r="K62" s="67"/>
+      <c r="K62" s="61"/>
       <c r="L62" s="40"/>
     </row>
     <row r="63" spans="1:12" s="52" customFormat="1" ht="24" x14ac:dyDescent="0.25">
@@ -3890,7 +4016,7 @@
       <c r="J63" s="40">
         <v>1</v>
       </c>
-      <c r="K63" s="80"/>
+      <c r="K63" s="74"/>
       <c r="L63" s="40"/>
     </row>
     <row r="64" spans="1:12" s="52" customFormat="1" ht="38.25" x14ac:dyDescent="0.25">
@@ -3923,7 +4049,7 @@
       <c r="J64" s="40">
         <v>1</v>
       </c>
-      <c r="K64" s="81" t="s">
+      <c r="K64" s="75" t="s">
         <v>270</v>
       </c>
       <c r="L64" s="40"/>
@@ -3958,7 +4084,7 @@
       <c r="J65" s="40">
         <v>1</v>
       </c>
-      <c r="K65" s="81" t="s">
+      <c r="K65" s="75" t="s">
         <v>270</v>
       </c>
       <c r="L65" s="40"/>
@@ -3991,7 +4117,7 @@
       <c r="J66" s="40">
         <v>1</v>
       </c>
-      <c r="K66" s="81" t="s">
+      <c r="K66" s="75" t="s">
         <v>270</v>
       </c>
       <c r="L66" s="40"/>
@@ -4026,7 +4152,7 @@
       <c r="J67" s="40">
         <v>1</v>
       </c>
-      <c r="K67" s="80"/>
+      <c r="K67" s="74"/>
       <c r="L67" s="59"/>
     </row>
     <row r="68" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -4040,41 +4166,330 @@
       <c r="H68" s="57"/>
       <c r="I68" s="58"/>
       <c r="J68" s="58"/>
-      <c r="K68" s="64"/>
-      <c r="L68" s="65"/>
-    </row>
-    <row r="73" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="K68" s="80"/>
+      <c r="L68" s="81"/>
+    </row>
+    <row r="71" spans="1:12" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="D71" s="86" t="s">
+        <v>308</v>
+      </c>
+      <c r="E71" s="86"/>
+      <c r="F71" s="86"/>
+      <c r="G71" s="86"/>
+    </row>
+    <row r="72" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="73" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A73" s="1"/>
+      <c r="B73" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="C73" s="27" t="s">
+        <v>6</v>
+      </c>
+      <c r="D73" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="E73" s="27" t="s">
+        <v>64</v>
+      </c>
+      <c r="F73" s="27" t="s">
+        <v>111</v>
+      </c>
+      <c r="G73" s="27" t="s">
+        <v>137</v>
+      </c>
+      <c r="H73" s="27" t="s">
+        <v>176</v>
+      </c>
+      <c r="I73" s="27" t="s">
+        <v>226</v>
+      </c>
+      <c r="J73" s="27" t="s">
+        <v>221</v>
+      </c>
+      <c r="K73" s="27" t="s">
+        <v>228</v>
+      </c>
+      <c r="L73" s="27" t="s">
+        <v>229</v>
+      </c>
     </row>
     <row r="74" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A74" s="1"/>
+      <c r="B74" s="34">
+        <v>1</v>
+      </c>
+      <c r="C74" s="82" t="s">
+        <v>7</v>
+      </c>
+      <c r="D74" s="33" t="s">
+        <v>277</v>
+      </c>
+      <c r="E74" s="33" t="s">
+        <v>278</v>
+      </c>
+      <c r="F74" s="33" t="s">
+        <v>114</v>
+      </c>
+      <c r="G74" s="33" t="s">
+        <v>279</v>
+      </c>
+      <c r="H74" s="33" t="s">
+        <v>280</v>
+      </c>
+      <c r="I74" s="33" t="s">
+        <v>281</v>
+      </c>
+      <c r="J74" s="33">
+        <v>4</v>
+      </c>
+      <c r="K74" s="33"/>
+      <c r="L74" s="83"/>
     </row>
     <row r="75" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A75" s="1"/>
+      <c r="B75" s="34">
+        <v>2</v>
+      </c>
+      <c r="C75" s="84" t="s">
+        <v>7</v>
+      </c>
+      <c r="D75" s="36" t="s">
+        <v>282</v>
+      </c>
+      <c r="E75" s="36" t="s">
+        <v>69</v>
+      </c>
+      <c r="F75" s="36" t="s">
+        <v>114</v>
+      </c>
+      <c r="G75" s="36" t="s">
+        <v>142</v>
+      </c>
+      <c r="H75" s="36" t="s">
+        <v>177</v>
+      </c>
+      <c r="I75" s="36" t="s">
+        <v>202</v>
+      </c>
+      <c r="J75" s="36">
+        <v>1</v>
+      </c>
+      <c r="K75" s="36"/>
+      <c r="L75" s="36"/>
     </row>
     <row r="76" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A76" s="1"/>
-    </row>
-    <row r="77" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="B76" s="34">
+        <v>3</v>
+      </c>
+      <c r="C76" s="82" t="s">
+        <v>8</v>
+      </c>
+      <c r="D76" s="33" t="s">
+        <v>283</v>
+      </c>
+      <c r="E76" s="33" t="s">
+        <v>284</v>
+      </c>
+      <c r="F76" s="33" t="s">
+        <v>285</v>
+      </c>
+      <c r="G76" s="33" t="s">
+        <v>286</v>
+      </c>
+      <c r="H76" s="33" t="s">
+        <v>287</v>
+      </c>
+      <c r="I76" s="33" t="s">
+        <v>223</v>
+      </c>
+      <c r="J76" s="33">
+        <v>1</v>
+      </c>
+      <c r="K76" s="33"/>
+      <c r="L76" s="40"/>
+    </row>
+    <row r="77" spans="1:12" ht="24" x14ac:dyDescent="0.25">
       <c r="A77" s="1"/>
-    </row>
-    <row r="78" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="B77" s="34">
+        <v>4</v>
+      </c>
+      <c r="C77" s="84" t="s">
+        <v>288</v>
+      </c>
+      <c r="D77" s="36" t="s">
+        <v>289</v>
+      </c>
+      <c r="E77" s="36" t="s">
+        <v>290</v>
+      </c>
+      <c r="F77" s="36" t="s">
+        <v>291</v>
+      </c>
+      <c r="G77" s="36" t="s">
+        <v>292</v>
+      </c>
+      <c r="H77" s="36" t="s">
+        <v>293</v>
+      </c>
+      <c r="I77" s="36" t="s">
+        <v>223</v>
+      </c>
+      <c r="J77" s="36">
+        <v>1</v>
+      </c>
+      <c r="K77" s="36"/>
+      <c r="L77" s="40"/>
+    </row>
+    <row r="78" spans="1:12" ht="48" x14ac:dyDescent="0.25">
       <c r="A78" s="1"/>
-    </row>
-    <row r="79" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="B78" s="34">
+        <v>5</v>
+      </c>
+      <c r="C78" s="82" t="s">
+        <v>248</v>
+      </c>
+      <c r="D78" s="33" t="s">
+        <v>35</v>
+      </c>
+      <c r="E78" s="33" t="s">
+        <v>250</v>
+      </c>
+      <c r="F78" s="33" t="s">
+        <v>224</v>
+      </c>
+      <c r="G78" s="33" t="s">
+        <v>251</v>
+      </c>
+      <c r="H78" s="33" t="s">
+        <v>247</v>
+      </c>
+      <c r="I78" s="33" t="s">
+        <v>223</v>
+      </c>
+      <c r="J78" s="33">
+        <v>1</v>
+      </c>
+      <c r="K78" s="33"/>
+      <c r="L78" s="40"/>
+    </row>
+    <row r="79" spans="1:12" ht="24" x14ac:dyDescent="0.25">
       <c r="A79" s="1"/>
+      <c r="B79" s="34">
+        <v>6</v>
+      </c>
+      <c r="C79" s="84" t="s">
+        <v>294</v>
+      </c>
+      <c r="D79" s="36" t="s">
+        <v>295</v>
+      </c>
+      <c r="E79" s="36" t="s">
+        <v>296</v>
+      </c>
+      <c r="F79" s="36" t="s">
+        <v>224</v>
+      </c>
+      <c r="G79" s="36" t="s">
+        <v>297</v>
+      </c>
+      <c r="H79" s="36" t="s">
+        <v>298</v>
+      </c>
+      <c r="I79" s="36" t="s">
+        <v>223</v>
+      </c>
+      <c r="J79" s="36">
+        <v>1</v>
+      </c>
+      <c r="K79" s="36"/>
+      <c r="L79" s="40"/>
     </row>
     <row r="80" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A80" s="1"/>
-    </row>
-    <row r="81" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B80" s="34">
+        <v>7</v>
+      </c>
+      <c r="C80" s="82" t="s">
+        <v>15</v>
+      </c>
+      <c r="D80" s="33" t="s">
+        <v>299</v>
+      </c>
+      <c r="E80" s="33" t="s">
+        <v>300</v>
+      </c>
+      <c r="F80" s="33" t="s">
+        <v>301</v>
+      </c>
+      <c r="G80" s="33" t="s">
+        <v>302</v>
+      </c>
+      <c r="H80" s="33" t="s">
+        <v>177</v>
+      </c>
+      <c r="I80" s="33" t="s">
+        <v>303</v>
+      </c>
+      <c r="J80" s="33">
+        <v>2</v>
+      </c>
+      <c r="K80" s="33"/>
+      <c r="L80" s="40"/>
+    </row>
+    <row r="81" spans="1:12" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A81" s="1"/>
+      <c r="B81" s="34">
+        <v>8</v>
+      </c>
+      <c r="C81" s="85" t="s">
+        <v>16</v>
+      </c>
+      <c r="D81" s="40" t="s">
+        <v>304</v>
+      </c>
+      <c r="E81" s="40" t="s">
+        <v>305</v>
+      </c>
+      <c r="F81" s="40" t="s">
+        <v>224</v>
+      </c>
+      <c r="G81" s="40" t="s">
+        <v>306</v>
+      </c>
+      <c r="H81" s="40" t="s">
+        <v>307</v>
+      </c>
+      <c r="I81" s="40" t="s">
+        <v>223</v>
+      </c>
+      <c r="J81" s="40">
+        <v>1</v>
+      </c>
+      <c r="K81" s="40"/>
+      <c r="L81" s="40"/>
+    </row>
+    <row r="82" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B82" s="53"/>
+      <c r="C82" s="54"/>
+      <c r="D82" s="55"/>
+      <c r="E82" s="56"/>
+      <c r="F82" s="57"/>
+      <c r="G82" s="58"/>
+      <c r="H82" s="57"/>
+      <c r="I82" s="58"/>
+      <c r="J82" s="58"/>
+      <c r="K82" s="80"/>
+      <c r="L82" s="81"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="5">
     <mergeCell ref="I1:L1"/>
     <mergeCell ref="L3:L8"/>
     <mergeCell ref="K68:L68"/>
+    <mergeCell ref="K82:L82"/>
+    <mergeCell ref="D71:G71"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -4113,11 +4528,11 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="60"/>
-      <c r="J1" s="60"/>
-      <c r="K1" s="60"/>
-      <c r="L1" s="60"/>
-      <c r="M1" s="61"/>
+      <c r="I1" s="76"/>
+      <c r="J1" s="76"/>
+      <c r="K1" s="76"/>
+      <c r="L1" s="76"/>
+      <c r="M1" s="77"/>
     </row>
     <row r="2" spans="1:13" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -4155,7 +4570,7 @@
       <c r="J3" s="5"/>
       <c r="K3" s="5"/>
       <c r="L3" s="5"/>
-      <c r="M3" s="62"/>
+      <c r="M3" s="78"/>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -4174,7 +4589,7 @@
       <c r="J4" s="6"/>
       <c r="K4" s="6"/>
       <c r="L4" s="6"/>
-      <c r="M4" s="63"/>
+      <c r="M4" s="79"/>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -4193,7 +4608,7 @@
       <c r="J5" s="6"/>
       <c r="K5" s="6"/>
       <c r="L5" s="6"/>
-      <c r="M5" s="63"/>
+      <c r="M5" s="79"/>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -4208,7 +4623,7 @@
       <c r="J6" s="6"/>
       <c r="K6" s="6"/>
       <c r="L6" s="6"/>
-      <c r="M6" s="63"/>
+      <c r="M6" s="79"/>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -4223,7 +4638,7 @@
       <c r="J7" s="8"/>
       <c r="K7" s="8"/>
       <c r="L7" s="8"/>
-      <c r="M7" s="63"/>
+      <c r="M7" s="79"/>
     </row>
     <row r="8" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -4238,7 +4653,7 @@
       <c r="J8" s="8"/>
       <c r="K8" s="8"/>
       <c r="L8" s="8"/>
-      <c r="M8" s="63"/>
+      <c r="M8" s="79"/>
     </row>
     <row r="9" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -4272,7 +4687,7 @@
       <c r="K9" s="27" t="s">
         <v>227</v>
       </c>
-      <c r="L9" s="66" t="s">
+      <c r="L9" s="60" t="s">
         <v>228</v>
       </c>
       <c r="M9" s="27" t="s">
@@ -4309,11 +4724,11 @@
       <c r="J10" s="33">
         <v>3</v>
       </c>
-      <c r="K10" s="67">
+      <c r="K10" s="61">
         <f>J10*5</f>
         <v>15</v>
       </c>
-      <c r="L10" s="67"/>
+      <c r="L10" s="61"/>
       <c r="M10" s="51"/>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
@@ -4346,11 +4761,11 @@
       <c r="J11" s="36">
         <v>2</v>
       </c>
-      <c r="K11" s="67">
+      <c r="K11" s="61">
         <f t="shared" ref="K11:K67" si="1">J11*5</f>
         <v>10</v>
       </c>
-      <c r="L11" s="68"/>
+      <c r="L11" s="62"/>
       <c r="M11" s="36"/>
     </row>
     <row r="12" spans="1:13" ht="24" x14ac:dyDescent="0.25">
@@ -4383,11 +4798,11 @@
       <c r="J12" s="33">
         <v>14</v>
       </c>
-      <c r="K12" s="67">
+      <c r="K12" s="61">
         <f t="shared" si="1"/>
         <v>70</v>
       </c>
-      <c r="L12" s="67"/>
+      <c r="L12" s="61"/>
       <c r="M12" s="40"/>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
@@ -4420,11 +4835,11 @@
       <c r="J13" s="36">
         <v>1</v>
       </c>
-      <c r="K13" s="67">
+      <c r="K13" s="61">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L13" s="68"/>
+      <c r="L13" s="62"/>
       <c r="M13" s="40"/>
     </row>
     <row r="14" spans="1:13" ht="48" x14ac:dyDescent="0.25">
@@ -4457,11 +4872,11 @@
       <c r="J14" s="33">
         <v>22</v>
       </c>
-      <c r="K14" s="67">
+      <c r="K14" s="61">
         <f t="shared" si="1"/>
         <v>110</v>
       </c>
-      <c r="L14" s="67"/>
+      <c r="L14" s="61"/>
       <c r="M14" s="40"/>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
@@ -4494,11 +4909,11 @@
       <c r="J15" s="36">
         <v>2</v>
       </c>
-      <c r="K15" s="67">
+      <c r="K15" s="61">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="L15" s="68"/>
+      <c r="L15" s="62"/>
       <c r="M15" s="40"/>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.25">
@@ -4531,11 +4946,11 @@
       <c r="J16" s="33">
         <v>2</v>
       </c>
-      <c r="K16" s="67">
+      <c r="K16" s="61">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="L16" s="67"/>
+      <c r="L16" s="61"/>
       <c r="M16" s="40"/>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.25">
@@ -4568,11 +4983,11 @@
       <c r="J17" s="36">
         <v>6</v>
       </c>
-      <c r="K17" s="67">
+      <c r="K17" s="61">
         <f t="shared" si="1"/>
         <v>30</v>
       </c>
-      <c r="L17" s="68"/>
+      <c r="L17" s="62"/>
       <c r="M17" s="40"/>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.25">
@@ -4605,11 +5020,11 @@
       <c r="J18" s="33">
         <v>3</v>
       </c>
-      <c r="K18" s="67">
+      <c r="K18" s="61">
         <f t="shared" si="1"/>
         <v>15</v>
       </c>
-      <c r="L18" s="67"/>
+      <c r="L18" s="61"/>
       <c r="M18" s="40"/>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.25">
@@ -4642,11 +5057,11 @@
       <c r="J19" s="36">
         <v>1</v>
       </c>
-      <c r="K19" s="67">
+      <c r="K19" s="61">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L19" s="68"/>
+      <c r="L19" s="62"/>
       <c r="M19" s="40"/>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.25">
@@ -4679,11 +5094,11 @@
       <c r="J20" s="36">
         <v>2</v>
       </c>
-      <c r="K20" s="67">
+      <c r="K20" s="61">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="L20" s="68"/>
+      <c r="L20" s="62"/>
       <c r="M20" s="40"/>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.25">
@@ -4716,11 +5131,11 @@
       <c r="J21" s="33">
         <v>2</v>
       </c>
-      <c r="K21" s="67">
+      <c r="K21" s="61">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="L21" s="67"/>
+      <c r="L21" s="61"/>
       <c r="M21" s="40"/>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.25">
@@ -4753,11 +5168,11 @@
       <c r="J22" s="36">
         <v>1</v>
       </c>
-      <c r="K22" s="67">
+      <c r="K22" s="61">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L22" s="68"/>
+      <c r="L22" s="62"/>
       <c r="M22" s="40"/>
     </row>
     <row r="23" spans="1:13" ht="24" x14ac:dyDescent="0.25">
@@ -4790,11 +5205,11 @@
       <c r="J23" s="36">
         <v>1</v>
       </c>
-      <c r="K23" s="67">
+      <c r="K23" s="61">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L23" s="68"/>
+      <c r="L23" s="62"/>
       <c r="M23" s="40"/>
     </row>
     <row r="24" spans="1:13" ht="24" x14ac:dyDescent="0.25">
@@ -4827,11 +5242,11 @@
       <c r="J24" s="33">
         <v>1</v>
       </c>
-      <c r="K24" s="67">
+      <c r="K24" s="61">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L24" s="67"/>
+      <c r="L24" s="61"/>
       <c r="M24" s="40"/>
     </row>
     <row r="25" spans="1:13" ht="24" x14ac:dyDescent="0.25">
@@ -4864,11 +5279,11 @@
       <c r="J25" s="36">
         <v>1</v>
       </c>
-      <c r="K25" s="67">
+      <c r="K25" s="61">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L25" s="69"/>
+      <c r="L25" s="63"/>
       <c r="M25" s="36"/>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.25">
@@ -4901,11 +5316,11 @@
       <c r="J26" s="33">
         <v>2</v>
       </c>
-      <c r="K26" s="67">
+      <c r="K26" s="61">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="L26" s="67"/>
+      <c r="L26" s="61"/>
       <c r="M26" s="40"/>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.25">
@@ -4938,11 +5353,11 @@
       <c r="J27" s="36">
         <v>1</v>
       </c>
-      <c r="K27" s="67">
+      <c r="K27" s="61">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L27" s="68"/>
+      <c r="L27" s="62"/>
       <c r="M27" s="40"/>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.25">
@@ -4975,11 +5390,11 @@
       <c r="J28" s="43">
         <v>1</v>
       </c>
-      <c r="K28" s="67">
+      <c r="K28" s="61">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L28" s="70"/>
+      <c r="L28" s="64"/>
       <c r="M28" s="46"/>
     </row>
     <row r="29" spans="1:13" ht="48" x14ac:dyDescent="0.25">
@@ -5012,11 +5427,11 @@
       <c r="J29" s="36">
         <v>3</v>
       </c>
-      <c r="K29" s="67">
+      <c r="K29" s="61">
         <f t="shared" si="1"/>
         <v>15</v>
       </c>
-      <c r="L29" s="68"/>
+      <c r="L29" s="62"/>
       <c r="M29" s="40"/>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.25">
@@ -5049,11 +5464,11 @@
       <c r="J30" s="33">
         <v>1</v>
       </c>
-      <c r="K30" s="67">
+      <c r="K30" s="61">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L30" s="71" t="s">
+      <c r="L30" s="65" t="s">
         <v>273</v>
       </c>
       <c r="M30" s="40"/>
@@ -5088,11 +5503,11 @@
       <c r="J31" s="36">
         <v>1</v>
       </c>
-      <c r="K31" s="67">
+      <c r="K31" s="61">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L31" s="68"/>
+      <c r="L31" s="62"/>
       <c r="M31" s="40"/>
     </row>
     <row r="32" spans="1:13" ht="48" x14ac:dyDescent="0.25">
@@ -5125,11 +5540,11 @@
       <c r="J32" s="33">
         <v>1</v>
       </c>
-      <c r="K32" s="67">
+      <c r="K32" s="61">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L32" s="67"/>
+      <c r="L32" s="61"/>
       <c r="M32" s="40"/>
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.25">
@@ -5162,11 +5577,11 @@
       <c r="J33" s="36">
         <v>1</v>
       </c>
-      <c r="K33" s="67">
+      <c r="K33" s="61">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L33" s="68"/>
+      <c r="L33" s="62"/>
       <c r="M33" s="40"/>
     </row>
     <row r="34" spans="1:13" ht="24" x14ac:dyDescent="0.25">
@@ -5199,11 +5614,11 @@
       <c r="J34" s="43">
         <v>13</v>
       </c>
-      <c r="K34" s="67">
+      <c r="K34" s="61">
         <f t="shared" si="1"/>
         <v>65</v>
       </c>
-      <c r="L34" s="70"/>
+      <c r="L34" s="64"/>
       <c r="M34" s="46"/>
     </row>
     <row r="35" spans="1:13" ht="36" x14ac:dyDescent="0.25">
@@ -5236,11 +5651,11 @@
       <c r="J35" s="36">
         <v>1</v>
       </c>
-      <c r="K35" s="67">
+      <c r="K35" s="61">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L35" s="68"/>
+      <c r="L35" s="62"/>
       <c r="M35" s="40"/>
     </row>
     <row r="36" spans="1:13" x14ac:dyDescent="0.25">
@@ -5273,11 +5688,11 @@
       <c r="J36" s="33">
         <v>1</v>
       </c>
-      <c r="K36" s="67">
+      <c r="K36" s="61">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L36" s="67"/>
+      <c r="L36" s="61"/>
       <c r="M36" s="40"/>
     </row>
     <row r="37" spans="1:13" ht="48" x14ac:dyDescent="0.25">
@@ -5310,11 +5725,11 @@
       <c r="J37" s="36">
         <v>11</v>
       </c>
-      <c r="K37" s="67">
+      <c r="K37" s="61">
         <f t="shared" si="1"/>
         <v>55</v>
       </c>
-      <c r="L37" s="72" t="s">
+      <c r="L37" s="66" t="s">
         <v>235</v>
       </c>
       <c r="M37" s="40"/>
@@ -5349,11 +5764,11 @@
       <c r="J38" s="36">
         <v>3</v>
       </c>
-      <c r="K38" s="67">
+      <c r="K38" s="61">
         <f t="shared" si="1"/>
         <v>15</v>
       </c>
-      <c r="L38" s="68"/>
+      <c r="L38" s="62"/>
       <c r="M38" s="40"/>
     </row>
     <row r="39" spans="1:13" x14ac:dyDescent="0.25">
@@ -5386,11 +5801,11 @@
       <c r="J39" s="36">
         <v>1</v>
       </c>
-      <c r="K39" s="67">
+      <c r="K39" s="61">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L39" s="67"/>
+      <c r="L39" s="61"/>
       <c r="M39" s="40"/>
     </row>
     <row r="40" spans="1:13" x14ac:dyDescent="0.25">
@@ -5423,11 +5838,11 @@
       <c r="J40" s="33">
         <v>2</v>
       </c>
-      <c r="K40" s="67">
+      <c r="K40" s="61">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="L40" s="67"/>
+      <c r="L40" s="61"/>
       <c r="M40" s="40"/>
     </row>
     <row r="41" spans="1:13" ht="24" x14ac:dyDescent="0.25">
@@ -5460,11 +5875,11 @@
       <c r="J41" s="36">
         <v>1</v>
       </c>
-      <c r="K41" s="67">
+      <c r="K41" s="61">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L41" s="68"/>
+      <c r="L41" s="62"/>
       <c r="M41" s="40"/>
     </row>
     <row r="42" spans="1:13" x14ac:dyDescent="0.25">
@@ -5497,11 +5912,11 @@
       <c r="J42" s="33">
         <v>5</v>
       </c>
-      <c r="K42" s="67">
+      <c r="K42" s="61">
         <f t="shared" si="1"/>
         <v>25</v>
       </c>
-      <c r="L42" s="67"/>
+      <c r="L42" s="61"/>
       <c r="M42" s="40"/>
     </row>
     <row r="43" spans="1:13" x14ac:dyDescent="0.25">
@@ -5534,11 +5949,11 @@
       <c r="J43" s="36">
         <v>2</v>
       </c>
-      <c r="K43" s="67">
+      <c r="K43" s="61">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="L43" s="68"/>
+      <c r="L43" s="62"/>
       <c r="M43" s="40"/>
     </row>
     <row r="44" spans="1:13" x14ac:dyDescent="0.25">
@@ -5571,11 +5986,11 @@
       <c r="J44" s="33">
         <v>3</v>
       </c>
-      <c r="K44" s="67">
+      <c r="K44" s="61">
         <f t="shared" si="1"/>
         <v>15</v>
       </c>
-      <c r="L44" s="67"/>
+      <c r="L44" s="61"/>
       <c r="M44" s="40"/>
     </row>
     <row r="45" spans="1:13" x14ac:dyDescent="0.25">
@@ -5608,11 +6023,11 @@
       <c r="J45" s="36">
         <v>2</v>
       </c>
-      <c r="K45" s="67">
+      <c r="K45" s="61">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="L45" s="68"/>
+      <c r="L45" s="62"/>
       <c r="M45" s="40"/>
     </row>
     <row r="46" spans="1:13" x14ac:dyDescent="0.25">
@@ -5645,49 +6060,49 @@
       <c r="J46" s="33">
         <v>2</v>
       </c>
-      <c r="K46" s="67">
+      <c r="K46" s="61">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="L46" s="67"/>
+      <c r="L46" s="61"/>
       <c r="M46" s="40"/>
     </row>
     <row r="47" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A47" s="73"/>
-      <c r="B47" s="74">
+      <c r="A47" s="67"/>
+      <c r="B47" s="68">
         <f t="shared" si="0"/>
         <v>38</v>
       </c>
-      <c r="C47" s="75" t="s">
+      <c r="C47" s="69" t="s">
         <v>15</v>
       </c>
-      <c r="D47" s="76" t="s">
+      <c r="D47" s="70" t="s">
         <v>51</v>
       </c>
-      <c r="E47" s="76" t="s">
+      <c r="E47" s="70" t="s">
         <v>96</v>
       </c>
-      <c r="F47" s="76" t="s">
+      <c r="F47" s="70" t="s">
         <v>123</v>
       </c>
-      <c r="G47" s="76" t="s">
+      <c r="G47" s="70" t="s">
         <v>163</v>
       </c>
-      <c r="H47" s="76" t="s">
+      <c r="H47" s="70" t="s">
         <v>177</v>
       </c>
-      <c r="I47" s="76" t="s">
+      <c r="I47" s="70" t="s">
         <v>219</v>
       </c>
-      <c r="J47" s="76">
-        <v>1</v>
-      </c>
-      <c r="K47" s="67">
+      <c r="J47" s="70">
+        <v>1</v>
+      </c>
+      <c r="K47" s="61">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L47" s="77"/>
-      <c r="M47" s="78"/>
+      <c r="L47" s="71"/>
+      <c r="M47" s="72"/>
     </row>
     <row r="48" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A48" s="50"/>
@@ -5719,11 +6134,11 @@
       <c r="J48" s="33">
         <v>1</v>
       </c>
-      <c r="K48" s="67">
+      <c r="K48" s="61">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L48" s="67"/>
+      <c r="L48" s="61"/>
       <c r="M48" s="40"/>
     </row>
     <row r="49" spans="1:13" x14ac:dyDescent="0.25">
@@ -5756,11 +6171,11 @@
       <c r="J49" s="43">
         <v>6</v>
       </c>
-      <c r="K49" s="67">
+      <c r="K49" s="61">
         <f t="shared" si="1"/>
         <v>30</v>
       </c>
-      <c r="L49" s="70"/>
+      <c r="L49" s="64"/>
       <c r="M49" s="46"/>
     </row>
     <row r="50" spans="1:13" ht="48" x14ac:dyDescent="0.25">
@@ -5793,11 +6208,11 @@
       <c r="J50" s="36">
         <v>2</v>
       </c>
-      <c r="K50" s="67">
+      <c r="K50" s="61">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="L50" s="72"/>
+      <c r="L50" s="66"/>
       <c r="M50" s="36"/>
     </row>
     <row r="51" spans="1:13" ht="36" x14ac:dyDescent="0.25">
@@ -5830,11 +6245,11 @@
       <c r="J51" s="33">
         <v>1</v>
       </c>
-      <c r="K51" s="67">
+      <c r="K51" s="61">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L51" s="79"/>
+      <c r="L51" s="73"/>
       <c r="M51" s="33"/>
     </row>
     <row r="52" spans="1:13" ht="48" x14ac:dyDescent="0.25">
@@ -5867,11 +6282,11 @@
       <c r="J52" s="36">
         <v>1</v>
       </c>
-      <c r="K52" s="67">
+      <c r="K52" s="61">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L52" s="68"/>
+      <c r="L52" s="62"/>
       <c r="M52" s="40"/>
     </row>
     <row r="53" spans="1:13" ht="24" x14ac:dyDescent="0.25">
@@ -5904,11 +6319,11 @@
       <c r="J53" s="33">
         <v>1</v>
       </c>
-      <c r="K53" s="67">
+      <c r="K53" s="61">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L53" s="67"/>
+      <c r="L53" s="61"/>
       <c r="M53" s="40"/>
     </row>
     <row r="54" spans="1:13" x14ac:dyDescent="0.25">
@@ -5941,11 +6356,11 @@
       <c r="J54" s="36">
         <v>1</v>
       </c>
-      <c r="K54" s="67">
+      <c r="K54" s="61">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L54" s="68"/>
+      <c r="L54" s="62"/>
       <c r="M54" s="40"/>
     </row>
     <row r="55" spans="1:13" x14ac:dyDescent="0.25">
@@ -5978,11 +6393,11 @@
       <c r="J55" s="33">
         <v>1</v>
       </c>
-      <c r="K55" s="67">
+      <c r="K55" s="61">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L55" s="67"/>
+      <c r="L55" s="61"/>
       <c r="M55" s="40"/>
     </row>
     <row r="56" spans="1:13" ht="24" x14ac:dyDescent="0.25">
@@ -6015,11 +6430,11 @@
       <c r="J56" s="36">
         <v>1</v>
       </c>
-      <c r="K56" s="67">
+      <c r="K56" s="61">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L56" s="68"/>
+      <c r="L56" s="62"/>
       <c r="M56" s="40"/>
     </row>
     <row r="57" spans="1:13" ht="24" x14ac:dyDescent="0.25">
@@ -6052,11 +6467,11 @@
       <c r="J57" s="33">
         <v>1</v>
       </c>
-      <c r="K57" s="67">
+      <c r="K57" s="61">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L57" s="67"/>
+      <c r="L57" s="61"/>
       <c r="M57" s="40"/>
     </row>
     <row r="58" spans="1:13" x14ac:dyDescent="0.25">
@@ -6089,11 +6504,11 @@
       <c r="J58" s="33">
         <v>1</v>
       </c>
-      <c r="K58" s="67">
+      <c r="K58" s="61">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L58" s="67"/>
+      <c r="L58" s="61"/>
       <c r="M58" s="40"/>
     </row>
     <row r="59" spans="1:13" ht="24" x14ac:dyDescent="0.25">
@@ -6126,11 +6541,11 @@
       <c r="J59" s="36">
         <v>1</v>
       </c>
-      <c r="K59" s="67">
+      <c r="K59" s="61">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L59" s="68"/>
+      <c r="L59" s="62"/>
       <c r="M59" s="40"/>
     </row>
     <row r="60" spans="1:13" ht="24" x14ac:dyDescent="0.25">
@@ -6163,11 +6578,11 @@
       <c r="J60" s="33">
         <v>1</v>
       </c>
-      <c r="K60" s="67">
+      <c r="K60" s="61">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L60" s="67"/>
+      <c r="L60" s="61"/>
       <c r="M60" s="40"/>
     </row>
     <row r="61" spans="1:13" x14ac:dyDescent="0.25">
@@ -6200,11 +6615,11 @@
       <c r="J61" s="36">
         <v>1</v>
       </c>
-      <c r="K61" s="67">
+      <c r="K61" s="61">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L61" s="68"/>
+      <c r="L61" s="62"/>
       <c r="M61" s="40"/>
     </row>
     <row r="62" spans="1:13" x14ac:dyDescent="0.25">
@@ -6237,11 +6652,11 @@
       <c r="J62" s="33">
         <v>1</v>
       </c>
-      <c r="K62" s="67">
+      <c r="K62" s="61">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L62" s="67"/>
+      <c r="L62" s="61"/>
       <c r="M62" s="40"/>
     </row>
     <row r="63" spans="1:13" ht="24" x14ac:dyDescent="0.25">
@@ -6274,11 +6689,11 @@
       <c r="J63" s="40">
         <v>1</v>
       </c>
-      <c r="K63" s="67">
+      <c r="K63" s="61">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L63" s="80"/>
+      <c r="L63" s="74"/>
       <c r="M63" s="40"/>
     </row>
     <row r="64" spans="1:13" ht="38.25" x14ac:dyDescent="0.25">
@@ -6311,11 +6726,11 @@
       <c r="J64" s="40">
         <v>1</v>
       </c>
-      <c r="K64" s="67">
+      <c r="K64" s="61">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L64" s="81" t="s">
+      <c r="L64" s="75" t="s">
         <v>270</v>
       </c>
       <c r="M64" s="40"/>
@@ -6350,11 +6765,11 @@
       <c r="J65" s="40">
         <v>1</v>
       </c>
-      <c r="K65" s="67">
+      <c r="K65" s="61">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L65" s="81" t="s">
+      <c r="L65" s="75" t="s">
         <v>270</v>
       </c>
       <c r="M65" s="40"/>
@@ -6387,11 +6802,11 @@
       <c r="J66" s="40">
         <v>1</v>
       </c>
-      <c r="K66" s="67">
+      <c r="K66" s="61">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L66" s="81" t="s">
+      <c r="L66" s="75" t="s">
         <v>270</v>
       </c>
       <c r="M66" s="40"/>
@@ -6426,11 +6841,11 @@
       <c r="J67" s="40">
         <v>1</v>
       </c>
-      <c r="K67" s="67">
+      <c r="K67" s="61">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L67" s="80"/>
+      <c r="L67" s="74"/>
       <c r="M67" s="59"/>
     </row>
     <row r="68" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -6445,8 +6860,8 @@
       <c r="I68" s="58"/>
       <c r="J68" s="58"/>
       <c r="K68" s="58"/>
-      <c r="L68" s="64"/>
-      <c r="M68" s="65"/>
+      <c r="L68" s="80"/>
+      <c r="M68" s="81"/>
     </row>
     <row r="69" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B69"/>

</xml_diff>

<commit_message>
minor change in client-BOM #9
</commit_message>
<xml_diff>
--- a/BOM/Client-BOM.xlsx
+++ b/BOM/Client-BOM.xlsx
@@ -5,7 +5,7 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\bryandelmee-olliealarm\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Faizan\GitHub\bryandelmee-olliealarm\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -15,12 +15,12 @@
     <sheet name="1 Board" sheetId="2" r:id="rId1"/>
     <sheet name="5 Boards" sheetId="1" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="152511"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="927" uniqueCount="309">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="886" uniqueCount="294">
   <si>
     <t>Component list</t>
   </si>
@@ -853,57 +853,6 @@
     <t>TS-1109S-C-B</t>
   </si>
   <si>
-    <t>C1, C2, C3, C4</t>
-  </si>
-  <si>
-    <t>CAP CER 1000PF 25V C0G 0402</t>
-  </si>
-  <si>
-    <t>C1005C0G1E102JT000F</t>
-  </si>
-  <si>
-    <t>TDK</t>
-  </si>
-  <si>
-    <t>1nF</t>
-  </si>
-  <si>
-    <t>C62</t>
-  </si>
-  <si>
-    <t>D1</t>
-  </si>
-  <si>
-    <t>TVS DIODE 5VWM 6.3VC DSN0603-2</t>
-  </si>
-  <si>
-    <t>DSN0603-2</t>
-  </si>
-  <si>
-    <t>PESD5V0H1BSFYL</t>
-  </si>
-  <si>
-    <t>Nexperia</t>
-  </si>
-  <si>
-    <t>Fuse</t>
-  </si>
-  <si>
-    <t>F1</t>
-  </si>
-  <si>
-    <t>6V 2A 50A 1W -40℃~+85℃ 4A 4mΩ 5s 45mΩ 0805 Resettable Fuses ROHS</t>
-  </si>
-  <si>
-    <t>Fuse-0805</t>
-  </si>
-  <si>
-    <t>BSMD0805L-200</t>
-  </si>
-  <si>
-    <t>BHFUSE</t>
-  </si>
-  <si>
     <t>USB Connector</t>
   </si>
   <si>
@@ -946,13 +895,19 @@
     <t>Korean Hroparts Elec</t>
   </si>
   <si>
-    <t>SIDE PCB BOM</t>
+    <t>Alarm-Clock-v1.1</t>
+  </si>
+  <si>
+    <t>Side-PCB-v1.1</t>
+  </si>
+  <si>
+    <t>Bill of Materials for Project Ollie-Alarm-Clock</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="[$-409]h:mm:ss\ AM/PM;@"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.0000"/>
@@ -1423,7 +1378,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="87">
+  <cellXfs count="86">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1626,6 +1581,15 @@
     <xf numFmtId="0" fontId="23" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="24" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1642,18 +1606,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1702,7 +1654,7 @@
         <xdr:cNvPr id="3" name="Picture 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1733,6 +1685,50 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>71</xdr:row>
+      <xdr:rowOff>10417</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1714500" cy="1104008"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="11410950" y="620017"/>
+          <a:ext cx="1714500" cy="1104008"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -1756,7 +1752,7 @@
         <xdr:cNvPr id="3" name="Picture 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2053,7 +2049,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L82"/>
+  <dimension ref="A1:L81"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3" bestFit="1" customWidth="1"/>
@@ -2078,10 +2074,10 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="76"/>
-      <c r="J1" s="76"/>
-      <c r="K1" s="76"/>
-      <c r="L1" s="77"/>
+      <c r="I1" s="79"/>
+      <c r="J1" s="79"/>
+      <c r="K1" s="79"/>
+      <c r="L1" s="80"/>
     </row>
     <row r="2" spans="1:12" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -2092,7 +2088,7 @@
       </c>
       <c r="E2" s="9"/>
       <c r="F2" s="37" t="s">
-        <v>230</v>
+        <v>293</v>
       </c>
       <c r="G2" s="10"/>
       <c r="H2" s="4"/>
@@ -2110,14 +2106,14 @@
       </c>
       <c r="E3" s="11"/>
       <c r="F3" s="38" t="s">
-        <v>231</v>
+        <v>291</v>
       </c>
       <c r="G3" s="11"/>
       <c r="H3" s="5"/>
       <c r="I3" s="5"/>
       <c r="J3" s="5"/>
       <c r="K3" s="5"/>
-      <c r="L3" s="78"/>
+      <c r="L3" s="81"/>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -2128,14 +2124,14 @@
       </c>
       <c r="E4" s="11"/>
       <c r="F4" s="38" t="s">
-        <v>231</v>
+        <v>291</v>
       </c>
       <c r="G4" s="12"/>
       <c r="H4" s="7"/>
       <c r="I4" s="7"/>
       <c r="J4" s="6"/>
       <c r="K4" s="6"/>
-      <c r="L4" s="79"/>
+      <c r="L4" s="82"/>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -2153,7 +2149,7 @@
       <c r="I5" s="6"/>
       <c r="J5" s="6"/>
       <c r="K5" s="6"/>
-      <c r="L5" s="79"/>
+      <c r="L5" s="82"/>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -2167,7 +2163,7 @@
       <c r="I6" s="6"/>
       <c r="J6" s="6"/>
       <c r="K6" s="6"/>
-      <c r="L6" s="79"/>
+      <c r="L6" s="82"/>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -2181,7 +2177,7 @@
       <c r="I7" s="8"/>
       <c r="J7" s="8"/>
       <c r="K7" s="8"/>
-      <c r="L7" s="79"/>
+      <c r="L7" s="82"/>
     </row>
     <row r="8" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -2195,7 +2191,7 @@
       <c r="I8" s="8"/>
       <c r="J8" s="8"/>
       <c r="K8" s="8"/>
-      <c r="L8" s="79"/>
+      <c r="L8" s="82"/>
     </row>
     <row r="9" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -2902,25 +2898,25 @@
       <c r="C30" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="D30" s="33" t="s">
+      <c r="D30" s="43" t="s">
         <v>36</v>
       </c>
-      <c r="E30" s="33" t="s">
+      <c r="E30" s="43" t="s">
         <v>82</v>
       </c>
-      <c r="F30" s="33" t="s">
+      <c r="F30" s="43" t="s">
         <v>224</v>
       </c>
-      <c r="G30" s="33" t="s">
+      <c r="G30" s="43" t="s">
         <v>119</v>
       </c>
-      <c r="H30" s="33" t="s">
+      <c r="H30" s="43" t="s">
         <v>183</v>
       </c>
-      <c r="I30" s="36" t="s">
-        <v>223</v>
-      </c>
-      <c r="J30" s="33">
+      <c r="I30" s="45" t="s">
+        <v>223</v>
+      </c>
+      <c r="J30" s="43">
         <v>1</v>
       </c>
       <c r="K30" s="65" t="s">
@@ -4166,330 +4162,241 @@
       <c r="H68" s="57"/>
       <c r="I68" s="58"/>
       <c r="J68" s="58"/>
-      <c r="K68" s="80"/>
-      <c r="L68" s="81"/>
-    </row>
-    <row r="71" spans="1:12" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="D71" s="86" t="s">
-        <v>308</v>
-      </c>
-      <c r="E71" s="86"/>
-      <c r="F71" s="86"/>
-      <c r="G71" s="86"/>
-    </row>
-    <row r="72" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="73" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K68" s="83"/>
+      <c r="L68" s="84"/>
+    </row>
+    <row r="70" spans="1:12" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D70" s="85"/>
+      <c r="E70" s="85"/>
+      <c r="F70" s="85"/>
+      <c r="G70" s="85"/>
+    </row>
+    <row r="71" spans="1:12" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B71" s="19"/>
+      <c r="C71" s="28"/>
+      <c r="D71" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="E71" s="9"/>
+      <c r="F71" s="37" t="s">
+        <v>293</v>
+      </c>
+      <c r="G71" s="10"/>
+      <c r="H71" s="4"/>
+      <c r="I71" s="4"/>
+      <c r="J71" s="4"/>
+      <c r="K71" s="4"/>
+      <c r="L71" s="3"/>
+    </row>
+    <row r="72" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A72" s="1"/>
+      <c r="B72" s="20"/>
+      <c r="C72" s="29"/>
+      <c r="D72" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="E72" s="11"/>
+      <c r="F72" s="38" t="s">
+        <v>292</v>
+      </c>
+      <c r="G72" s="11"/>
+      <c r="H72" s="5"/>
+      <c r="I72" s="5"/>
+      <c r="J72" s="5"/>
+      <c r="K72" s="5"/>
+      <c r="L72" s="81"/>
+    </row>
+    <row r="73" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A73" s="1"/>
-      <c r="B73" s="27" t="s">
-        <v>4</v>
-      </c>
-      <c r="C73" s="27" t="s">
-        <v>6</v>
-      </c>
-      <c r="D73" s="27" t="s">
-        <v>19</v>
-      </c>
-      <c r="E73" s="27" t="s">
-        <v>64</v>
-      </c>
-      <c r="F73" s="27" t="s">
-        <v>111</v>
-      </c>
-      <c r="G73" s="27" t="s">
-        <v>137</v>
-      </c>
-      <c r="H73" s="27" t="s">
-        <v>176</v>
-      </c>
-      <c r="I73" s="27" t="s">
-        <v>226</v>
-      </c>
-      <c r="J73" s="27" t="s">
-        <v>221</v>
-      </c>
-      <c r="K73" s="27" t="s">
-        <v>228</v>
-      </c>
-      <c r="L73" s="27" t="s">
-        <v>229</v>
-      </c>
+      <c r="B73" s="20"/>
+      <c r="C73" s="29"/>
+      <c r="D73" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="E73" s="11"/>
+      <c r="F73" s="38" t="s">
+        <v>292</v>
+      </c>
+      <c r="G73" s="12"/>
+      <c r="H73" s="7"/>
+      <c r="I73" s="7"/>
+      <c r="J73" s="6"/>
+      <c r="K73" s="6"/>
+      <c r="L73" s="82"/>
     </row>
     <row r="74" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A74" s="1"/>
-      <c r="B74" s="34">
-        <v>1</v>
-      </c>
-      <c r="C74" s="82" t="s">
-        <v>7</v>
-      </c>
-      <c r="D74" s="33" t="s">
-        <v>277</v>
-      </c>
-      <c r="E74" s="33" t="s">
-        <v>278</v>
-      </c>
-      <c r="F74" s="33" t="s">
-        <v>114</v>
-      </c>
-      <c r="G74" s="33" t="s">
-        <v>279</v>
-      </c>
-      <c r="H74" s="33" t="s">
-        <v>280</v>
-      </c>
-      <c r="I74" s="33" t="s">
-        <v>281</v>
-      </c>
-      <c r="J74" s="33">
-        <v>4</v>
-      </c>
-      <c r="K74" s="33"/>
-      <c r="L74" s="83"/>
+      <c r="B74" s="20"/>
+      <c r="C74" s="29"/>
+      <c r="D74" s="11"/>
+      <c r="E74" s="11"/>
+      <c r="F74" s="39"/>
+      <c r="G74" s="13"/>
+      <c r="H74" s="6"/>
+      <c r="I74" s="6"/>
+      <c r="J74" s="6"/>
+      <c r="K74" s="6"/>
+      <c r="L74" s="82"/>
     </row>
     <row r="75" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A75" s="1"/>
-      <c r="B75" s="34">
-        <v>2</v>
-      </c>
-      <c r="C75" s="84" t="s">
-        <v>7</v>
-      </c>
-      <c r="D75" s="36" t="s">
-        <v>282</v>
-      </c>
-      <c r="E75" s="36" t="s">
-        <v>69</v>
-      </c>
-      <c r="F75" s="36" t="s">
-        <v>114</v>
-      </c>
-      <c r="G75" s="36" t="s">
-        <v>142</v>
-      </c>
-      <c r="H75" s="36" t="s">
-        <v>177</v>
-      </c>
-      <c r="I75" s="36" t="s">
-        <v>202</v>
-      </c>
-      <c r="J75" s="36">
-        <v>1</v>
-      </c>
-      <c r="K75" s="36"/>
-      <c r="L75" s="36"/>
+      <c r="B75" s="21"/>
+      <c r="C75" s="30"/>
+      <c r="D75" s="14"/>
+      <c r="E75" s="14"/>
+      <c r="F75" s="15"/>
+      <c r="G75" s="13"/>
+      <c r="H75" s="6"/>
+      <c r="I75" s="6"/>
+      <c r="J75" s="6"/>
+      <c r="K75" s="6"/>
+      <c r="L75" s="82"/>
     </row>
     <row r="76" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A76" s="1"/>
-      <c r="B76" s="34">
-        <v>3</v>
-      </c>
-      <c r="C76" s="82" t="s">
-        <v>8</v>
-      </c>
-      <c r="D76" s="33" t="s">
-        <v>283</v>
-      </c>
-      <c r="E76" s="33" t="s">
-        <v>284</v>
-      </c>
-      <c r="F76" s="33" t="s">
-        <v>285</v>
-      </c>
-      <c r="G76" s="33" t="s">
-        <v>286</v>
-      </c>
-      <c r="H76" s="33" t="s">
-        <v>287</v>
-      </c>
-      <c r="I76" s="33" t="s">
-        <v>223</v>
-      </c>
-      <c r="J76" s="33">
-        <v>1</v>
-      </c>
-      <c r="K76" s="33"/>
-      <c r="L76" s="40"/>
-    </row>
-    <row r="77" spans="1:12" ht="24" x14ac:dyDescent="0.25">
+      <c r="B76" s="22"/>
+      <c r="C76" s="31"/>
+      <c r="D76" s="16"/>
+      <c r="E76" s="16"/>
+      <c r="F76" s="17"/>
+      <c r="G76" s="16"/>
+      <c r="H76" s="8"/>
+      <c r="I76" s="8"/>
+      <c r="J76" s="8"/>
+      <c r="K76" s="8"/>
+      <c r="L76" s="82"/>
+    </row>
+    <row r="77" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A77" s="1"/>
-      <c r="B77" s="34">
-        <v>4</v>
-      </c>
-      <c r="C77" s="84" t="s">
-        <v>288</v>
-      </c>
-      <c r="D77" s="36" t="s">
-        <v>289</v>
-      </c>
-      <c r="E77" s="36" t="s">
-        <v>290</v>
-      </c>
-      <c r="F77" s="36" t="s">
-        <v>291</v>
-      </c>
-      <c r="G77" s="36" t="s">
-        <v>292</v>
-      </c>
-      <c r="H77" s="36" t="s">
-        <v>293</v>
-      </c>
-      <c r="I77" s="36" t="s">
-        <v>223</v>
-      </c>
-      <c r="J77" s="36">
-        <v>1</v>
-      </c>
-      <c r="K77" s="36"/>
-      <c r="L77" s="40"/>
-    </row>
-    <row r="78" spans="1:12" ht="48" x14ac:dyDescent="0.25">
+      <c r="B77" s="24"/>
+      <c r="C77" s="32"/>
+      <c r="D77" s="25"/>
+      <c r="E77" s="25"/>
+      <c r="F77" s="26"/>
+      <c r="G77" s="16"/>
+      <c r="H77" s="8"/>
+      <c r="I77" s="8"/>
+      <c r="J77" s="8"/>
+      <c r="K77" s="8"/>
+      <c r="L77" s="82"/>
+    </row>
+    <row r="78" spans="1:12" ht="24" x14ac:dyDescent="0.25">
       <c r="A78" s="1"/>
       <c r="B78" s="34">
-        <v>5</v>
-      </c>
-      <c r="C78" s="82" t="s">
-        <v>248</v>
-      </c>
-      <c r="D78" s="33" t="s">
-        <v>35</v>
-      </c>
-      <c r="E78" s="33" t="s">
-        <v>250</v>
-      </c>
-      <c r="F78" s="33" t="s">
+        <v>6</v>
+      </c>
+      <c r="C78" s="77" t="s">
+        <v>277</v>
+      </c>
+      <c r="D78" s="36" t="s">
+        <v>278</v>
+      </c>
+      <c r="E78" s="36" t="s">
+        <v>279</v>
+      </c>
+      <c r="F78" s="36" t="s">
         <v>224</v>
       </c>
-      <c r="G78" s="33" t="s">
-        <v>251</v>
-      </c>
-      <c r="H78" s="33" t="s">
-        <v>247</v>
-      </c>
-      <c r="I78" s="33" t="s">
-        <v>223</v>
-      </c>
-      <c r="J78" s="33">
-        <v>1</v>
-      </c>
-      <c r="K78" s="33"/>
+      <c r="G78" s="36" t="s">
+        <v>280</v>
+      </c>
+      <c r="H78" s="36" t="s">
+        <v>281</v>
+      </c>
+      <c r="I78" s="36" t="s">
+        <v>223</v>
+      </c>
+      <c r="J78" s="36">
+        <v>1</v>
+      </c>
+      <c r="K78" s="36"/>
       <c r="L78" s="40"/>
     </row>
-    <row r="79" spans="1:12" ht="24" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A79" s="1"/>
       <c r="B79" s="34">
-        <v>6</v>
-      </c>
-      <c r="C79" s="84" t="s">
-        <v>294</v>
-      </c>
-      <c r="D79" s="36" t="s">
-        <v>295</v>
-      </c>
-      <c r="E79" s="36" t="s">
-        <v>296</v>
-      </c>
-      <c r="F79" s="36" t="s">
-        <v>224</v>
-      </c>
-      <c r="G79" s="36" t="s">
-        <v>297</v>
-      </c>
-      <c r="H79" s="36" t="s">
-        <v>298</v>
-      </c>
-      <c r="I79" s="36" t="s">
-        <v>223</v>
-      </c>
-      <c r="J79" s="36">
-        <v>1</v>
-      </c>
-      <c r="K79" s="36"/>
+        <v>7</v>
+      </c>
+      <c r="C79" s="76" t="s">
+        <v>15</v>
+      </c>
+      <c r="D79" s="33" t="s">
+        <v>282</v>
+      </c>
+      <c r="E79" s="33" t="s">
+        <v>283</v>
+      </c>
+      <c r="F79" s="33" t="s">
+        <v>284</v>
+      </c>
+      <c r="G79" s="33" t="s">
+        <v>285</v>
+      </c>
+      <c r="H79" s="33" t="s">
+        <v>177</v>
+      </c>
+      <c r="I79" s="33" t="s">
+        <v>286</v>
+      </c>
+      <c r="J79" s="33">
+        <v>2</v>
+      </c>
+      <c r="K79" s="33"/>
       <c r="L79" s="40"/>
     </row>
-    <row r="80" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:12" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A80" s="1"/>
       <c r="B80" s="34">
-        <v>7</v>
-      </c>
-      <c r="C80" s="82" t="s">
-        <v>15</v>
-      </c>
-      <c r="D80" s="33" t="s">
-        <v>299</v>
-      </c>
-      <c r="E80" s="33" t="s">
-        <v>300</v>
-      </c>
-      <c r="F80" s="33" t="s">
-        <v>301</v>
-      </c>
-      <c r="G80" s="33" t="s">
-        <v>302</v>
-      </c>
-      <c r="H80" s="33" t="s">
-        <v>177</v>
-      </c>
-      <c r="I80" s="33" t="s">
-        <v>303</v>
-      </c>
-      <c r="J80" s="33">
-        <v>2</v>
-      </c>
-      <c r="K80" s="33"/>
+        <v>8</v>
+      </c>
+      <c r="C80" s="78" t="s">
+        <v>16</v>
+      </c>
+      <c r="D80" s="40" t="s">
+        <v>287</v>
+      </c>
+      <c r="E80" s="40" t="s">
+        <v>288</v>
+      </c>
+      <c r="F80" s="40" t="s">
+        <v>224</v>
+      </c>
+      <c r="G80" s="40" t="s">
+        <v>289</v>
+      </c>
+      <c r="H80" s="40" t="s">
+        <v>290</v>
+      </c>
+      <c r="I80" s="40" t="s">
+        <v>223</v>
+      </c>
+      <c r="J80" s="40">
+        <v>1</v>
+      </c>
+      <c r="K80" s="40"/>
       <c r="L80" s="40"/>
     </row>
-    <row r="81" spans="1:12" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A81" s="1"/>
-      <c r="B81" s="34">
-        <v>8</v>
-      </c>
-      <c r="C81" s="85" t="s">
-        <v>16</v>
-      </c>
-      <c r="D81" s="40" t="s">
-        <v>304</v>
-      </c>
-      <c r="E81" s="40" t="s">
-        <v>305</v>
-      </c>
-      <c r="F81" s="40" t="s">
-        <v>224</v>
-      </c>
-      <c r="G81" s="40" t="s">
-        <v>306</v>
-      </c>
-      <c r="H81" s="40" t="s">
-        <v>307</v>
-      </c>
-      <c r="I81" s="40" t="s">
-        <v>223</v>
-      </c>
-      <c r="J81" s="40">
-        <v>1</v>
-      </c>
-      <c r="K81" s="40"/>
-      <c r="L81" s="40"/>
-    </row>
-    <row r="82" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B82" s="53"/>
-      <c r="C82" s="54"/>
-      <c r="D82" s="55"/>
-      <c r="E82" s="56"/>
-      <c r="F82" s="57"/>
-      <c r="G82" s="58"/>
-      <c r="H82" s="57"/>
-      <c r="I82" s="58"/>
-      <c r="J82" s="58"/>
-      <c r="K82" s="80"/>
-      <c r="L82" s="81"/>
+    <row r="81" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B81" s="53"/>
+      <c r="C81" s="54"/>
+      <c r="D81" s="55"/>
+      <c r="E81" s="56"/>
+      <c r="F81" s="57"/>
+      <c r="G81" s="58"/>
+      <c r="H81" s="57"/>
+      <c r="I81" s="58"/>
+      <c r="J81" s="58"/>
+      <c r="K81" s="83"/>
+      <c r="L81" s="84"/>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="6">
     <mergeCell ref="I1:L1"/>
     <mergeCell ref="L3:L8"/>
     <mergeCell ref="K68:L68"/>
-    <mergeCell ref="K82:L82"/>
-    <mergeCell ref="D71:G71"/>
+    <mergeCell ref="K81:L81"/>
+    <mergeCell ref="D70:G70"/>
+    <mergeCell ref="L72:L77"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -4528,11 +4435,11 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="76"/>
-      <c r="J1" s="76"/>
-      <c r="K1" s="76"/>
-      <c r="L1" s="76"/>
-      <c r="M1" s="77"/>
+      <c r="I1" s="79"/>
+      <c r="J1" s="79"/>
+      <c r="K1" s="79"/>
+      <c r="L1" s="79"/>
+      <c r="M1" s="80"/>
     </row>
     <row r="2" spans="1:13" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -4570,7 +4477,7 @@
       <c r="J3" s="5"/>
       <c r="K3" s="5"/>
       <c r="L3" s="5"/>
-      <c r="M3" s="78"/>
+      <c r="M3" s="81"/>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -4589,7 +4496,7 @@
       <c r="J4" s="6"/>
       <c r="K4" s="6"/>
       <c r="L4" s="6"/>
-      <c r="M4" s="79"/>
+      <c r="M4" s="82"/>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -4608,7 +4515,7 @@
       <c r="J5" s="6"/>
       <c r="K5" s="6"/>
       <c r="L5" s="6"/>
-      <c r="M5" s="79"/>
+      <c r="M5" s="82"/>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -4623,7 +4530,7 @@
       <c r="J6" s="6"/>
       <c r="K6" s="6"/>
       <c r="L6" s="6"/>
-      <c r="M6" s="79"/>
+      <c r="M6" s="82"/>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -4638,7 +4545,7 @@
       <c r="J7" s="8"/>
       <c r="K7" s="8"/>
       <c r="L7" s="8"/>
-      <c r="M7" s="79"/>
+      <c r="M7" s="82"/>
     </row>
     <row r="8" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -4653,7 +4560,7 @@
       <c r="J8" s="8"/>
       <c r="K8" s="8"/>
       <c r="L8" s="8"/>
-      <c r="M8" s="79"/>
+      <c r="M8" s="82"/>
     </row>
     <row r="9" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -6860,8 +6767,8 @@
       <c r="I68" s="58"/>
       <c r="J68" s="58"/>
       <c r="K68" s="58"/>
-      <c r="L68" s="80"/>
-      <c r="M68" s="81"/>
+      <c r="L68" s="83"/>
+      <c r="M68" s="84"/>
     </row>
     <row r="69" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B69"/>

</xml_diff>